<commit_message>
feat: Add directory-only version of update_records_list with simplified column mapping and noise statistics extraction
- Introduced `update_records_list_v6.py` for processing JSON metadata and data files from a specified directory.
- Simplified column mapping for header extraction.
- Ensured `h_nz_frac` and `ml_nz_frac` are always treated as percentages.
- Implemented noise statistics calculation and ectopy detection within the new script.
- Added command-line arguments for denoising and ectopy configuration paths.
- Enhanced Excel output with updated noise statistics and parameters.
</commit_message>
<xml_diff>
--- a/0_SELECT_ZIVE_DATA_2023/AtsisiuntimasZiveDuomenu/DuomenysTestui/zive_irasai_testui_isplestas.xlsx
+++ b/0_SELECT_ZIVE_DATA_2023/AtsisiuntimasZiveDuomenu/DuomenysTestui/zive_irasai_testui_isplestas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kesju\DI\2025_ZIVEO\PROJECT_TRAIN_UNET\0_SELECT_ZIVE_DATA_2023\AtsisiuntimasZiveDuomenu\DuomenysTestui\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DD66499-9010-462E-BD78-28CF3E282284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B909C0-B064-4E11-A3EE-9EF5B46620FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="93">
   <si>
     <t>filename</t>
   </si>
@@ -312,6 +312,9 @@
   </si>
   <si>
     <t>ectU</t>
+  </si>
+  <si>
+    <t>Notes</t>
   </si>
 </sst>
 </file>
@@ -1911,7 +1914,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5226947-0C6C-41DD-89DC-9E5D5CCC7401}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>